<commit_message>
Bieu Mau Bai Lieu
</commit_message>
<xml_diff>
--- a/public/TagDongCoVoi.xlsx
+++ b/public/TagDongCoVoi.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47452A83-E7B3-4BC8-A9B4-28DC440C1AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="4"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoVoi1" sheetId="1" r:id="rId1"/>
@@ -905,9 +906,6 @@
     <t>AI_2#_small_kiln_pier_lubricant_temperature_display</t>
   </si>
   <si>
-    <t>AI_3#_small_kiln_pier_lubricant_temperature_displa</t>
-  </si>
-  <si>
     <t>AI_4#_small_kiln_pier_lubricant_temperature_display</t>
   </si>
   <si>
@@ -987,12 +985,15 @@
   </si>
   <si>
     <t>Kiln_Behind_bearing_temperature_of_the_cooling_blower_motor</t>
+  </si>
+  <si>
+    <t>AI_3#_small_kiln_pier_lubricant_temperature_display</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1164,7 +1165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1182,18 +1183,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1201,8 +1195,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1224,16 +1225,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1514,7 +1505,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1542,10 +1533,10 @@
       <c r="E1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F1" s="16">
-        <v>135</v>
-      </c>
-      <c r="G1" s="11">
+      <c r="F1" s="6">
+        <v>135</v>
+      </c>
+      <c r="G1" s="6">
         <v>145</v>
       </c>
     </row>
@@ -1563,10 +1554,10 @@
       <c r="E2" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F2" s="16">
-        <v>135</v>
-      </c>
-      <c r="G2" s="11">
+      <c r="F2" s="6">
+        <v>135</v>
+      </c>
+      <c r="G2" s="6">
         <v>145</v>
       </c>
     </row>
@@ -1584,10 +1575,10 @@
       <c r="E3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F3" s="16">
-        <v>135</v>
-      </c>
-      <c r="G3" s="11">
+      <c r="F3" s="6">
+        <v>135</v>
+      </c>
+      <c r="G3" s="6">
         <v>145</v>
       </c>
     </row>
@@ -1605,10 +1596,10 @@
       <c r="E4" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F4" s="16">
-        <v>90</v>
-      </c>
-      <c r="G4" s="11">
+      <c r="F4" s="6">
+        <v>90</v>
+      </c>
+      <c r="G4" s="6">
         <v>95</v>
       </c>
     </row>
@@ -1626,10 +1617,10 @@
       <c r="E5" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F5" s="16">
-        <v>90</v>
-      </c>
-      <c r="G5" s="11">
+      <c r="F5" s="6">
+        <v>90</v>
+      </c>
+      <c r="G5" s="6">
         <v>95</v>
       </c>
     </row>
@@ -1647,10 +1638,10 @@
       <c r="E6" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F6" s="16">
-        <v>90</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="F6" s="6">
+        <v>90</v>
+      </c>
+      <c r="G6" s="6">
         <v>95</v>
       </c>
     </row>
@@ -1668,52 +1659,52 @@
       <c r="E7" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="16">
-        <v>90</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="F7" s="6">
+        <v>90</v>
+      </c>
+      <c r="G7" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="18"/>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="13">
         <v>8</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="19"/>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F9" s="24">
+      <c r="F9" s="13">
         <v>8</v>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="13">
         <v>11</v>
       </c>
     </row>
@@ -1733,7 +1724,7 @@
       <c r="E10" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="6">
         <v>135</v>
       </c>
       <c r="G10" s="6">
@@ -1754,7 +1745,7 @@
       <c r="E11" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="6">
         <v>135</v>
       </c>
       <c r="G11" s="6">
@@ -1775,7 +1766,7 @@
       <c r="E12" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="6">
         <v>135</v>
       </c>
       <c r="G12" s="6">
@@ -1796,7 +1787,7 @@
       <c r="E13" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="6">
         <v>90</v>
       </c>
       <c r="G13" s="6">
@@ -1817,7 +1808,7 @@
       <c r="E14" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="6">
         <v>90</v>
       </c>
       <c r="G14" s="6">
@@ -1838,7 +1829,7 @@
       <c r="E15" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="6">
         <v>90</v>
       </c>
       <c r="G15" s="6">
@@ -1859,7 +1850,7 @@
       <c r="E16" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="6">
         <v>90</v>
       </c>
       <c r="G16" s="6">
@@ -1868,43 +1859,43 @@
     </row>
     <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="18"/>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="13">
         <v>8</v>
       </c>
-      <c r="G17" s="24">
+      <c r="G17" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="19"/>
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="26" t="s">
+      <c r="C18" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="13">
         <v>8</v>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="13">
         <v>11</v>
       </c>
     </row>
@@ -1924,7 +1915,7 @@
       <c r="E19" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="6">
         <v>135</v>
       </c>
       <c r="G19" s="6">
@@ -1945,10 +1936,10 @@
       <c r="E20" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F20" s="16">
-        <v>135</v>
-      </c>
-      <c r="G20" s="11">
+      <c r="F20" s="6">
+        <v>135</v>
+      </c>
+      <c r="G20" s="6">
         <v>145</v>
       </c>
     </row>
@@ -1966,10 +1957,10 @@
       <c r="E21" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F21" s="16">
-        <v>135</v>
-      </c>
-      <c r="G21" s="11">
+      <c r="F21" s="6">
+        <v>135</v>
+      </c>
+      <c r="G21" s="6">
         <v>145</v>
       </c>
     </row>
@@ -1987,7 +1978,7 @@
       <c r="E22" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="6">
         <v>90</v>
       </c>
       <c r="G22" s="6">
@@ -2008,10 +1999,10 @@
       <c r="E23" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F23" s="16">
-        <v>90</v>
-      </c>
-      <c r="G23" s="11">
+      <c r="F23" s="6">
+        <v>90</v>
+      </c>
+      <c r="G23" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2029,10 +2020,10 @@
       <c r="E24" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F24" s="16">
-        <v>90</v>
-      </c>
-      <c r="G24" s="11">
+      <c r="F24" s="6">
+        <v>90</v>
+      </c>
+      <c r="G24" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2050,52 +2041,52 @@
       <c r="E25" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F25" s="16">
-        <v>90</v>
-      </c>
-      <c r="G25" s="11">
+      <c r="F25" s="6">
+        <v>90</v>
+      </c>
+      <c r="G25" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="18"/>
-      <c r="B26" s="25" t="s">
+      <c r="B26" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="D26" s="26" t="s">
+      <c r="D26" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="E26" s="26" t="s">
+      <c r="E26" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F26" s="24">
+      <c r="F26" s="13">
         <v>8</v>
       </c>
-      <c r="G26" s="24">
+      <c r="G26" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="19"/>
-      <c r="B27" s="25" t="s">
+      <c r="B27" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="D27" s="26" t="s">
+      <c r="D27" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="E27" s="26" t="s">
+      <c r="E27" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F27" s="24">
+      <c r="F27" s="13">
         <v>8</v>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="13">
         <v>11</v>
       </c>
     </row>
@@ -2115,10 +2106,10 @@
       <c r="E28" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="16">
-        <v>135</v>
-      </c>
-      <c r="G28" s="11">
+      <c r="F28" s="6">
+        <v>135</v>
+      </c>
+      <c r="G28" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2136,10 +2127,10 @@
       <c r="E29" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F29" s="16">
-        <v>135</v>
-      </c>
-      <c r="G29" s="11">
+      <c r="F29" s="6">
+        <v>135</v>
+      </c>
+      <c r="G29" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2157,10 +2148,10 @@
       <c r="E30" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F30" s="16">
-        <v>135</v>
-      </c>
-      <c r="G30" s="11">
+      <c r="F30" s="6">
+        <v>135</v>
+      </c>
+      <c r="G30" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2178,10 +2169,10 @@
       <c r="E31" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F31" s="16">
-        <v>90</v>
-      </c>
-      <c r="G31" s="11">
+      <c r="F31" s="6">
+        <v>90</v>
+      </c>
+      <c r="G31" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2199,10 +2190,10 @@
       <c r="E32" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F32" s="16">
-        <v>90</v>
-      </c>
-      <c r="G32" s="11">
+      <c r="F32" s="6">
+        <v>90</v>
+      </c>
+      <c r="G32" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2220,10 +2211,10 @@
       <c r="E33" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F33" s="16">
-        <v>90</v>
-      </c>
-      <c r="G33" s="11">
+      <c r="F33" s="6">
+        <v>90</v>
+      </c>
+      <c r="G33" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2241,56 +2232,56 @@
       <c r="E34" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F34" s="16">
-        <v>90</v>
-      </c>
-      <c r="G34" s="11">
+      <c r="F34" s="6">
+        <v>90</v>
+      </c>
+      <c r="G34" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="20"/>
-      <c r="B35" s="25" t="s">
+      <c r="B35" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C35" s="26" t="s">
+      <c r="C35" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D35" s="26" t="s">
+      <c r="D35" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="E35" s="26" t="s">
+      <c r="E35" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F35" s="24">
+      <c r="F35" s="13">
         <v>8</v>
       </c>
-      <c r="G35" s="24">
+      <c r="G35" s="13">
         <v>11</v>
       </c>
-      <c r="H35" s="15"/>
+      <c r="H35" s="12"/>
     </row>
     <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="20"/>
-      <c r="B36" s="25" t="s">
+      <c r="B36" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C36" s="26" t="s">
+      <c r="C36" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="D36" s="26" t="s">
+      <c r="D36" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="26" t="s">
+      <c r="E36" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F36" s="24">
+      <c r="F36" s="13">
         <v>8</v>
       </c>
-      <c r="G36" s="24">
+      <c r="G36" s="13">
         <v>11</v>
       </c>
-      <c r="H36" s="15"/>
+      <c r="H36" s="12"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="F37" s="6" t="s">
@@ -2313,7 +2304,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2342,10 +2333,10 @@
       <c r="E1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F1" s="16">
-        <v>135</v>
-      </c>
-      <c r="G1" s="11">
+      <c r="F1" s="6">
+        <v>135</v>
+      </c>
+      <c r="G1" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2363,10 +2354,10 @@
       <c r="E2" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F2" s="16">
-        <v>135</v>
-      </c>
-      <c r="G2" s="11">
+      <c r="F2" s="6">
+        <v>135</v>
+      </c>
+      <c r="G2" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2384,10 +2375,10 @@
       <c r="E3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F3" s="16">
-        <v>135</v>
-      </c>
-      <c r="G3" s="11">
+      <c r="F3" s="6">
+        <v>135</v>
+      </c>
+      <c r="G3" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2405,10 +2396,10 @@
       <c r="E4" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F4" s="16">
-        <v>90</v>
-      </c>
-      <c r="G4" s="11">
+      <c r="F4" s="6">
+        <v>90</v>
+      </c>
+      <c r="G4" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2426,10 +2417,10 @@
       <c r="E5" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F5" s="16">
-        <v>90</v>
-      </c>
-      <c r="G5" s="11">
+      <c r="F5" s="6">
+        <v>90</v>
+      </c>
+      <c r="G5" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2447,10 +2438,10 @@
       <c r="E6" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F6" s="16">
-        <v>90</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="F6" s="6">
+        <v>90</v>
+      </c>
+      <c r="G6" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2468,31 +2459,31 @@
       <c r="E7" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="16">
-        <v>90</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="F7" s="6">
+        <v>90</v>
+      </c>
+      <c r="G7" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="20"/>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="13">
         <v>8</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="13">
         <v>11</v>
       </c>
     </row>
@@ -2512,10 +2503,10 @@
       <c r="E9" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F9" s="16">
-        <v>135</v>
-      </c>
-      <c r="G9" s="11">
+      <c r="F9" s="6">
+        <v>135</v>
+      </c>
+      <c r="G9" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2533,10 +2524,10 @@
       <c r="E10" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F10" s="16">
-        <v>135</v>
-      </c>
-      <c r="G10" s="11">
+      <c r="F10" s="6">
+        <v>135</v>
+      </c>
+      <c r="G10" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2554,10 +2545,10 @@
       <c r="E11" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F11" s="16">
-        <v>135</v>
-      </c>
-      <c r="G11" s="11">
+      <c r="F11" s="6">
+        <v>135</v>
+      </c>
+      <c r="G11" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2575,10 +2566,10 @@
       <c r="E12" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F12" s="16">
-        <v>90</v>
-      </c>
-      <c r="G12" s="11">
+      <c r="F12" s="6">
+        <v>90</v>
+      </c>
+      <c r="G12" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2596,10 +2587,10 @@
       <c r="E13" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F13" s="16">
-        <v>90</v>
-      </c>
-      <c r="G13" s="11">
+      <c r="F13" s="6">
+        <v>90</v>
+      </c>
+      <c r="G13" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2617,10 +2608,10 @@
       <c r="E14" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F14" s="16">
-        <v>90</v>
-      </c>
-      <c r="G14" s="11">
+      <c r="F14" s="6">
+        <v>90</v>
+      </c>
+      <c r="G14" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2638,31 +2629,31 @@
       <c r="E15" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F15" s="16">
-        <v>90</v>
-      </c>
-      <c r="G15" s="11">
+      <c r="F15" s="6">
+        <v>90</v>
+      </c>
+      <c r="G15" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="20"/>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="D16" s="26" t="s">
+      <c r="D16" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="13">
         <v>8</v>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="13">
         <v>11</v>
       </c>
     </row>
@@ -2682,10 +2673,10 @@
       <c r="E17" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F17" s="16">
-        <v>135</v>
-      </c>
-      <c r="G17" s="11">
+      <c r="F17" s="6">
+        <v>135</v>
+      </c>
+      <c r="G17" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2703,10 +2694,10 @@
       <c r="E18" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F18" s="16">
-        <v>135</v>
-      </c>
-      <c r="G18" s="11">
+      <c r="F18" s="6">
+        <v>135</v>
+      </c>
+      <c r="G18" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2724,10 +2715,10 @@
       <c r="E19" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F19" s="16">
-        <v>135</v>
-      </c>
-      <c r="G19" s="11">
+      <c r="F19" s="6">
+        <v>135</v>
+      </c>
+      <c r="G19" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2745,10 +2736,10 @@
       <c r="E20" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F20" s="16">
-        <v>90</v>
-      </c>
-      <c r="G20" s="11">
+      <c r="F20" s="6">
+        <v>90</v>
+      </c>
+      <c r="G20" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2766,10 +2757,10 @@
       <c r="E21" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F21" s="16">
-        <v>90</v>
-      </c>
-      <c r="G21" s="11">
+      <c r="F21" s="6">
+        <v>90</v>
+      </c>
+      <c r="G21" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2787,10 +2778,10 @@
       <c r="E22" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F22" s="16">
-        <v>90</v>
-      </c>
-      <c r="G22" s="11">
+      <c r="F22" s="6">
+        <v>90</v>
+      </c>
+      <c r="G22" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2808,52 +2799,52 @@
       <c r="E23" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F23" s="16">
-        <v>90</v>
-      </c>
-      <c r="G23" s="11">
+      <c r="F23" s="6">
+        <v>90</v>
+      </c>
+      <c r="G23" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="20"/>
-      <c r="B24" s="25" t="s">
+      <c r="B24" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="26" t="s">
+      <c r="C24" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="26" t="s">
+      <c r="E24" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F24" s="24">
+      <c r="F24" s="13">
         <v>8</v>
       </c>
-      <c r="G24" s="24">
+      <c r="G24" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="20"/>
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="26" t="s">
+      <c r="C25" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="E25" s="26" t="s">
+      <c r="E25" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F25" s="24">
+      <c r="F25" s="13">
         <v>8</v>
       </c>
-      <c r="G25" s="24">
+      <c r="G25" s="13">
         <v>11</v>
       </c>
     </row>
@@ -2873,10 +2864,10 @@
       <c r="E26" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F26" s="16">
-        <v>135</v>
-      </c>
-      <c r="G26" s="11">
+      <c r="F26" s="6">
+        <v>135</v>
+      </c>
+      <c r="G26" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2894,10 +2885,10 @@
       <c r="E27" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F27" s="16">
-        <v>135</v>
-      </c>
-      <c r="G27" s="11">
+      <c r="F27" s="6">
+        <v>135</v>
+      </c>
+      <c r="G27" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2915,10 +2906,10 @@
       <c r="E28" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="16">
-        <v>135</v>
-      </c>
-      <c r="G28" s="11">
+      <c r="F28" s="6">
+        <v>135</v>
+      </c>
+      <c r="G28" s="6">
         <v>145</v>
       </c>
     </row>
@@ -2936,10 +2927,10 @@
       <c r="E29" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F29" s="16">
-        <v>90</v>
-      </c>
-      <c r="G29" s="11">
+      <c r="F29" s="6">
+        <v>90</v>
+      </c>
+      <c r="G29" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2957,10 +2948,10 @@
       <c r="E30" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F30" s="16">
-        <v>90</v>
-      </c>
-      <c r="G30" s="11">
+      <c r="F30" s="6">
+        <v>90</v>
+      </c>
+      <c r="G30" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2978,10 +2969,10 @@
       <c r="E31" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F31" s="16">
-        <v>90</v>
-      </c>
-      <c r="G31" s="11">
+      <c r="F31" s="6">
+        <v>90</v>
+      </c>
+      <c r="G31" s="6">
         <v>95</v>
       </c>
     </row>
@@ -2999,52 +2990,52 @@
       <c r="E32" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F32" s="16">
-        <v>90</v>
-      </c>
-      <c r="G32" s="11">
+      <c r="F32" s="6">
+        <v>90</v>
+      </c>
+      <c r="G32" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="20"/>
-      <c r="B33" s="25" t="s">
+      <c r="B33" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="C33" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="D33" s="26" t="s">
+      <c r="D33" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="E33" s="26" t="s">
+      <c r="E33" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F33" s="24">
+      <c r="F33" s="13">
         <v>8</v>
       </c>
-      <c r="G33" s="24">
+      <c r="G33" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="20"/>
-      <c r="B34" s="25" t="s">
+      <c r="B34" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C34" s="26" t="s">
+      <c r="C34" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="D34" s="26" t="s">
+      <c r="D34" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E34" s="26" t="s">
+      <c r="E34" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F34" s="24">
+      <c r="F34" s="13">
         <v>8</v>
       </c>
-      <c r="G34" s="24">
+      <c r="G34" s="13">
         <v>11</v>
       </c>
     </row>
@@ -3068,7 +3059,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3097,10 +3088,10 @@
       <c r="E1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F1" s="16">
-        <v>135</v>
-      </c>
-      <c r="G1" s="11">
+      <c r="F1" s="6">
+        <v>135</v>
+      </c>
+      <c r="G1" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3118,10 +3109,10 @@
       <c r="E2" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F2" s="16">
-        <v>135</v>
-      </c>
-      <c r="G2" s="11">
+      <c r="F2" s="6">
+        <v>135</v>
+      </c>
+      <c r="G2" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3139,10 +3130,10 @@
       <c r="E3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F3" s="16">
-        <v>135</v>
-      </c>
-      <c r="G3" s="11">
+      <c r="F3" s="6">
+        <v>135</v>
+      </c>
+      <c r="G3" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3160,10 +3151,10 @@
       <c r="E4" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F4" s="16">
-        <v>90</v>
-      </c>
-      <c r="G4" s="11">
+      <c r="F4" s="6">
+        <v>90</v>
+      </c>
+      <c r="G4" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3181,10 +3172,10 @@
       <c r="E5" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F5" s="16">
-        <v>90</v>
-      </c>
-      <c r="G5" s="11">
+      <c r="F5" s="6">
+        <v>90</v>
+      </c>
+      <c r="G5" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3202,10 +3193,10 @@
       <c r="E6" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F6" s="16">
-        <v>90</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="F6" s="6">
+        <v>90</v>
+      </c>
+      <c r="G6" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3223,31 +3214,31 @@
       <c r="E7" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="16">
-        <v>90</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="F7" s="6">
+        <v>90</v>
+      </c>
+      <c r="G7" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="20"/>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="E8" s="26" t="s">
+      <c r="D8" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="13">
         <v>8</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="13">
         <v>11</v>
       </c>
     </row>
@@ -3267,10 +3258,10 @@
       <c r="E9" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F9" s="16">
-        <v>135</v>
-      </c>
-      <c r="G9" s="11">
+      <c r="F9" s="6">
+        <v>135</v>
+      </c>
+      <c r="G9" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3288,10 +3279,10 @@
       <c r="E10" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F10" s="16">
-        <v>135</v>
-      </c>
-      <c r="G10" s="11">
+      <c r="F10" s="6">
+        <v>135</v>
+      </c>
+      <c r="G10" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3309,10 +3300,10 @@
       <c r="E11" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F11" s="16">
-        <v>135</v>
-      </c>
-      <c r="G11" s="11">
+      <c r="F11" s="6">
+        <v>135</v>
+      </c>
+      <c r="G11" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3330,10 +3321,10 @@
       <c r="E12" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F12" s="16">
-        <v>90</v>
-      </c>
-      <c r="G12" s="11">
+      <c r="F12" s="6">
+        <v>90</v>
+      </c>
+      <c r="G12" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3351,10 +3342,10 @@
       <c r="E13" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F13" s="16">
-        <v>90</v>
-      </c>
-      <c r="G13" s="11">
+      <c r="F13" s="6">
+        <v>90</v>
+      </c>
+      <c r="G13" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3372,10 +3363,10 @@
       <c r="E14" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F14" s="16">
-        <v>90</v>
-      </c>
-      <c r="G14" s="11">
+      <c r="F14" s="6">
+        <v>90</v>
+      </c>
+      <c r="G14" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3393,31 +3384,31 @@
       <c r="E15" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F15" s="16">
-        <v>90</v>
-      </c>
-      <c r="G15" s="11">
+      <c r="F15" s="6">
+        <v>90</v>
+      </c>
+      <c r="G15" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="20"/>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="D16" s="26" t="s">
+      <c r="D16" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="13">
         <v>8</v>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="13">
         <v>11</v>
       </c>
     </row>
@@ -3437,10 +3428,10 @@
       <c r="E17" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F17" s="16">
-        <v>135</v>
-      </c>
-      <c r="G17" s="11">
+      <c r="F17" s="6">
+        <v>135</v>
+      </c>
+      <c r="G17" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3458,10 +3449,10 @@
       <c r="E18" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F18" s="16">
-        <v>135</v>
-      </c>
-      <c r="G18" s="11">
+      <c r="F18" s="6">
+        <v>135</v>
+      </c>
+      <c r="G18" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3479,10 +3470,10 @@
       <c r="E19" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F19" s="16">
-        <v>135</v>
-      </c>
-      <c r="G19" s="11">
+      <c r="F19" s="6">
+        <v>135</v>
+      </c>
+      <c r="G19" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3500,10 +3491,10 @@
       <c r="E20" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F20" s="16">
-        <v>90</v>
-      </c>
-      <c r="G20" s="11">
+      <c r="F20" s="6">
+        <v>90</v>
+      </c>
+      <c r="G20" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3521,10 +3512,10 @@
       <c r="E21" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F21" s="16">
-        <v>90</v>
-      </c>
-      <c r="G21" s="11">
+      <c r="F21" s="6">
+        <v>90</v>
+      </c>
+      <c r="G21" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3542,10 +3533,10 @@
       <c r="E22" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F22" s="16">
-        <v>90</v>
-      </c>
-      <c r="G22" s="11">
+      <c r="F22" s="6">
+        <v>90</v>
+      </c>
+      <c r="G22" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3563,52 +3554,52 @@
       <c r="E23" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F23" s="16">
-        <v>90</v>
-      </c>
-      <c r="G23" s="11">
+      <c r="F23" s="6">
+        <v>90</v>
+      </c>
+      <c r="G23" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="20"/>
-      <c r="B24" s="25" t="s">
+      <c r="B24" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="26" t="s">
+      <c r="C24" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="E24" s="26" t="s">
+      <c r="E24" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F24" s="24">
+      <c r="F24" s="13">
         <v>8</v>
       </c>
-      <c r="G24" s="24">
+      <c r="G24" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="20"/>
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="26" t="s">
+      <c r="C25" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="E25" s="26" t="s">
+      <c r="E25" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F25" s="24">
+      <c r="F25" s="13">
         <v>8</v>
       </c>
-      <c r="G25" s="24">
+      <c r="G25" s="13">
         <v>11</v>
       </c>
     </row>
@@ -3628,10 +3619,10 @@
       <c r="E26" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F26" s="16">
-        <v>135</v>
-      </c>
-      <c r="G26" s="11">
+      <c r="F26" s="6">
+        <v>135</v>
+      </c>
+      <c r="G26" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3649,10 +3640,10 @@
       <c r="E27" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F27" s="16">
-        <v>135</v>
-      </c>
-      <c r="G27" s="11">
+      <c r="F27" s="6">
+        <v>135</v>
+      </c>
+      <c r="G27" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3670,10 +3661,10 @@
       <c r="E28" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="16">
-        <v>135</v>
-      </c>
-      <c r="G28" s="11">
+      <c r="F28" s="6">
+        <v>135</v>
+      </c>
+      <c r="G28" s="6">
         <v>145</v>
       </c>
     </row>
@@ -3691,10 +3682,10 @@
       <c r="E29" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F29" s="16">
-        <v>90</v>
-      </c>
-      <c r="G29" s="11">
+      <c r="F29" s="6">
+        <v>90</v>
+      </c>
+      <c r="G29" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3712,10 +3703,10 @@
       <c r="E30" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F30" s="16">
-        <v>90</v>
-      </c>
-      <c r="G30" s="11">
+      <c r="F30" s="6">
+        <v>90</v>
+      </c>
+      <c r="G30" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3733,10 +3724,10 @@
       <c r="E31" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F31" s="16">
-        <v>90</v>
-      </c>
-      <c r="G31" s="11">
+      <c r="F31" s="6">
+        <v>90</v>
+      </c>
+      <c r="G31" s="6">
         <v>95</v>
       </c>
     </row>
@@ -3754,52 +3745,52 @@
       <c r="E32" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F32" s="16">
-        <v>90</v>
-      </c>
-      <c r="G32" s="11">
+      <c r="F32" s="6">
+        <v>90</v>
+      </c>
+      <c r="G32" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="20"/>
-      <c r="B33" s="25" t="s">
+      <c r="B33" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="C33" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="D33" s="26" t="s">
+      <c r="D33" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="E33" s="26" t="s">
+      <c r="E33" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F33" s="24">
+      <c r="F33" s="13">
         <v>8</v>
       </c>
-      <c r="G33" s="24">
+      <c r="G33" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="20"/>
-      <c r="B34" s="25" t="s">
+      <c r="B34" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C34" s="26" t="s">
+      <c r="C34" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="D34" s="26" t="s">
+      <c r="D34" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="E34" s="26" t="s">
+      <c r="E34" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F34" s="24">
+      <c r="F34" s="13">
         <v>8</v>
       </c>
-      <c r="G34" s="24">
+      <c r="G34" s="13">
         <v>11</v>
       </c>
     </row>
@@ -3823,7 +3814,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3840,7 +3831,7 @@
       <c r="A1" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -3855,13 +3846,13 @@
       <c r="F1" s="6">
         <v>135</v>
       </c>
-      <c r="G1" s="11">
+      <c r="G1" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="18"/>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -3873,16 +3864,16 @@
       <c r="E2" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F2" s="16">
-        <v>135</v>
-      </c>
-      <c r="G2" s="11">
+      <c r="F2" s="6">
+        <v>135</v>
+      </c>
+      <c r="G2" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="18"/>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -3894,16 +3885,16 @@
       <c r="E3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F3" s="16">
-        <v>135</v>
-      </c>
-      <c r="G3" s="11">
+      <c r="F3" s="6">
+        <v>135</v>
+      </c>
+      <c r="G3" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="18"/>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -3918,13 +3909,13 @@
       <c r="F4" s="6">
         <v>90</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="18"/>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -3936,16 +3927,16 @@
       <c r="E5" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F5" s="16">
-        <v>90</v>
-      </c>
-      <c r="G5" s="11">
+      <c r="F5" s="6">
+        <v>90</v>
+      </c>
+      <c r="G5" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="18"/>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -3957,16 +3948,16 @@
       <c r="E6" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F6" s="16">
-        <v>90</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="F6" s="6">
+        <v>90</v>
+      </c>
+      <c r="G6" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="18"/>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -3978,52 +3969,52 @@
       <c r="E7" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="16">
-        <v>90</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="F7" s="6">
+        <v>90</v>
+      </c>
+      <c r="G7" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="18"/>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="13">
         <v>8</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="19"/>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F9" s="24">
+      <c r="F9" s="13">
         <v>8</v>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="13">
         <v>11</v>
       </c>
     </row>
@@ -4031,7 +4022,7 @@
       <c r="A10" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -4043,16 +4034,16 @@
       <c r="E10" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F10" s="16">
-        <v>135</v>
-      </c>
-      <c r="G10" s="11">
+      <c r="F10" s="6">
+        <v>135</v>
+      </c>
+      <c r="G10" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="18"/>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -4064,16 +4055,16 @@
       <c r="E11" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F11" s="16">
-        <v>135</v>
-      </c>
-      <c r="G11" s="11">
+      <c r="F11" s="6">
+        <v>135</v>
+      </c>
+      <c r="G11" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="18"/>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -4085,16 +4076,16 @@
       <c r="E12" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F12" s="16">
-        <v>135</v>
-      </c>
-      <c r="G12" s="11">
+      <c r="F12" s="6">
+        <v>135</v>
+      </c>
+      <c r="G12" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="18"/>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -4106,58 +4097,58 @@
       <c r="E13" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F13" s="16">
-        <v>90</v>
-      </c>
-      <c r="G13" s="11">
+      <c r="F13" s="6">
+        <v>90</v>
+      </c>
+      <c r="G13" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="18"/>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>138</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F14" s="16">
-        <v>90</v>
-      </c>
-      <c r="G14" s="11">
+      <c r="F14" s="6">
+        <v>90</v>
+      </c>
+      <c r="G14" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="18"/>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="15" t="s">
         <v>180</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F15" s="16">
-        <v>90</v>
-      </c>
-      <c r="G15" s="11">
+      <c r="F15" s="6">
+        <v>90</v>
+      </c>
+      <c r="G15" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="18"/>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -4169,52 +4160,52 @@
       <c r="E16" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F16" s="16">
-        <v>90</v>
-      </c>
-      <c r="G16" s="11">
+      <c r="F16" s="6">
+        <v>90</v>
+      </c>
+      <c r="G16" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="18"/>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="13">
         <v>8</v>
       </c>
-      <c r="G17" s="24">
+      <c r="G17" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="19"/>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="26" t="s">
+      <c r="C18" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="13">
         <v>8</v>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="13">
         <v>11</v>
       </c>
     </row>
@@ -4222,7 +4213,7 @@
       <c r="A19" s="20" t="s">
         <v>184</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -4234,16 +4225,16 @@
       <c r="E19" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F19" s="16">
-        <v>135</v>
-      </c>
-      <c r="G19" s="11">
+      <c r="F19" s="6">
+        <v>135</v>
+      </c>
+      <c r="G19" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="20"/>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -4255,16 +4246,16 @@
       <c r="E20" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F20" s="16">
-        <v>135</v>
-      </c>
-      <c r="G20" s="11">
+      <c r="F20" s="6">
+        <v>135</v>
+      </c>
+      <c r="G20" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="20"/>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -4276,16 +4267,16 @@
       <c r="E21" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F21" s="16">
-        <v>135</v>
-      </c>
-      <c r="G21" s="11">
+      <c r="F21" s="6">
+        <v>135</v>
+      </c>
+      <c r="G21" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="20"/>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -4297,16 +4288,16 @@
       <c r="E22" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F22" s="16">
-        <v>90</v>
-      </c>
-      <c r="G22" s="11">
+      <c r="F22" s="6">
+        <v>90</v>
+      </c>
+      <c r="G22" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="20"/>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -4318,16 +4309,16 @@
       <c r="E23" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F23" s="16">
-        <v>90</v>
-      </c>
-      <c r="G23" s="11">
+      <c r="F23" s="6">
+        <v>90</v>
+      </c>
+      <c r="G23" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="20"/>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -4339,16 +4330,16 @@
       <c r="E24" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F24" s="16">
-        <v>90</v>
-      </c>
-      <c r="G24" s="11">
+      <c r="F24" s="6">
+        <v>90</v>
+      </c>
+      <c r="G24" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="20"/>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -4360,52 +4351,52 @@
       <c r="E25" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F25" s="16">
-        <v>90</v>
-      </c>
-      <c r="G25" s="11">
+      <c r="F25" s="6">
+        <v>90</v>
+      </c>
+      <c r="G25" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="20"/>
-      <c r="B26" s="27" t="s">
+      <c r="B26" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="D26" s="26" t="s">
+      <c r="D26" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="E26" s="26" t="s">
+      <c r="E26" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F26" s="24">
+      <c r="F26" s="13">
         <v>8</v>
       </c>
-      <c r="G26" s="24">
+      <c r="G26" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="20"/>
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="D27" s="26" t="s">
+      <c r="D27" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="E27" s="26" t="s">
+      <c r="E27" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F27" s="24">
+      <c r="F27" s="13">
         <v>8</v>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="13">
         <v>11</v>
       </c>
     </row>
@@ -4413,7 +4404,7 @@
       <c r="A28" s="20" t="s">
         <v>194</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -4425,16 +4416,16 @@
       <c r="E28" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="16">
-        <v>135</v>
-      </c>
-      <c r="G28" s="11">
+      <c r="F28" s="6">
+        <v>135</v>
+      </c>
+      <c r="G28" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="20"/>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -4446,16 +4437,16 @@
       <c r="E29" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F29" s="16">
-        <v>135</v>
-      </c>
-      <c r="G29" s="11">
+      <c r="F29" s="6">
+        <v>135</v>
+      </c>
+      <c r="G29" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="20"/>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -4467,16 +4458,16 @@
       <c r="E30" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F30" s="16">
-        <v>135</v>
-      </c>
-      <c r="G30" s="11">
+      <c r="F30" s="6">
+        <v>135</v>
+      </c>
+      <c r="G30" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="20"/>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -4488,16 +4479,16 @@
       <c r="E31" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F31" s="16">
-        <v>90</v>
-      </c>
-      <c r="G31" s="11">
+      <c r="F31" s="6">
+        <v>90</v>
+      </c>
+      <c r="G31" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="20"/>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -4509,16 +4500,16 @@
       <c r="E32" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F32" s="16">
-        <v>90</v>
-      </c>
-      <c r="G32" s="11">
+      <c r="F32" s="6">
+        <v>90</v>
+      </c>
+      <c r="G32" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="20"/>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -4530,16 +4521,16 @@
       <c r="E33" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F33" s="16">
-        <v>90</v>
-      </c>
-      <c r="G33" s="11">
+      <c r="F33" s="6">
+        <v>90</v>
+      </c>
+      <c r="G33" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="20"/>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -4551,52 +4542,52 @@
       <c r="E34" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F34" s="16">
-        <v>90</v>
-      </c>
-      <c r="G34" s="11">
+      <c r="F34" s="6">
+        <v>90</v>
+      </c>
+      <c r="G34" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="20"/>
-      <c r="B35" s="27" t="s">
+      <c r="B35" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C35" s="26" t="s">
+      <c r="C35" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D35" s="26" t="s">
+      <c r="D35" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="E35" s="26" t="s">
+      <c r="E35" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F35" s="24">
+      <c r="F35" s="13">
         <v>8</v>
       </c>
-      <c r="G35" s="24">
+      <c r="G35" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="20"/>
-      <c r="B36" s="27" t="s">
+      <c r="B36" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C36" s="26" t="s">
+      <c r="C36" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="D36" s="26" t="s">
+      <c r="D36" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="E36" s="26" t="s">
+      <c r="E36" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F36" s="24">
+      <c r="F36" s="13">
         <v>8</v>
       </c>
-      <c r="G36" s="24">
+      <c r="G36" s="13">
         <v>11</v>
       </c>
     </row>
@@ -4604,190 +4595,190 @@
       <c r="A37" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="D37" s="2" t="s">
         <v>205</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F37" s="16">
-        <v>135</v>
-      </c>
-      <c r="G37" s="11">
+      <c r="F37" s="6">
+        <v>135</v>
+      </c>
+      <c r="G37" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="20"/>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="2" t="s">
         <v>206</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F38" s="16">
-        <v>135</v>
-      </c>
-      <c r="G38" s="11">
+      <c r="F38" s="6">
+        <v>135</v>
+      </c>
+      <c r="G38" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="20"/>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="D39" s="9" t="s">
+      <c r="D39" s="2" t="s">
         <v>207</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F39" s="16">
-        <v>135</v>
-      </c>
-      <c r="G39" s="11">
+      <c r="F39" s="6">
+        <v>135</v>
+      </c>
+      <c r="G39" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="20"/>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="D40" s="2" t="s">
         <v>208</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F40" s="16">
-        <v>90</v>
-      </c>
-      <c r="G40" s="11">
+      <c r="F40" s="6">
+        <v>90</v>
+      </c>
+      <c r="G40" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="20"/>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="D41" s="9" t="s">
+      <c r="D41" s="2" t="s">
         <v>209</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F41" s="16">
-        <v>90</v>
-      </c>
-      <c r="G41" s="11">
+      <c r="F41" s="6">
+        <v>90</v>
+      </c>
+      <c r="G41" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="20"/>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="D42" s="2" t="s">
         <v>210</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F42" s="16">
-        <v>90</v>
-      </c>
-      <c r="G42" s="11">
+      <c r="F42" s="6">
+        <v>90</v>
+      </c>
+      <c r="G42" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="20"/>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="2" t="s">
         <v>211</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F43" s="16">
-        <v>90</v>
-      </c>
-      <c r="G43" s="11">
+      <c r="F43" s="6">
+        <v>90</v>
+      </c>
+      <c r="G43" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="20"/>
-      <c r="B44" s="27" t="s">
+      <c r="B44" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C44" s="26" t="s">
+      <c r="C44" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="D44" s="26" t="s">
+      <c r="D44" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="E44" s="26" t="s">
+      <c r="E44" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F44" s="24">
+      <c r="F44" s="13">
         <v>8</v>
       </c>
-      <c r="G44" s="24">
+      <c r="G44" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="20"/>
-      <c r="B45" s="27" t="s">
+      <c r="B45" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C45" s="26" t="s">
+      <c r="C45" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="D45" s="26" t="s">
+      <c r="D45" s="15" t="s">
         <v>213</v>
       </c>
-      <c r="E45" s="26" t="s">
+      <c r="E45" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F45" s="24">
+      <c r="F45" s="13">
         <v>8</v>
       </c>
-      <c r="G45" s="24">
+      <c r="G45" s="13">
         <v>11</v>
       </c>
     </row>
@@ -4813,7 +4804,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4827,7 +4818,7 @@
       <c r="A1" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -4839,16 +4830,16 @@
       <c r="E1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F1" s="16">
-        <v>135</v>
-      </c>
-      <c r="G1" s="11">
+      <c r="F1" s="6">
+        <v>135</v>
+      </c>
+      <c r="G1" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="20"/>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -4860,16 +4851,16 @@
       <c r="E2" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F2" s="16">
-        <v>135</v>
-      </c>
-      <c r="G2" s="11">
+      <c r="F2" s="6">
+        <v>135</v>
+      </c>
+      <c r="G2" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="20"/>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -4881,16 +4872,16 @@
       <c r="E3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F3" s="16">
-        <v>135</v>
-      </c>
-      <c r="G3" s="11">
+      <c r="F3" s="6">
+        <v>135</v>
+      </c>
+      <c r="G3" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="20"/>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -4902,16 +4893,16 @@
       <c r="E4" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F4" s="16">
-        <v>90</v>
-      </c>
-      <c r="G4" s="11">
+      <c r="F4" s="6">
+        <v>90</v>
+      </c>
+      <c r="G4" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="20"/>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -4923,16 +4914,16 @@
       <c r="E5" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F5" s="16">
-        <v>90</v>
-      </c>
-      <c r="G5" s="11">
+      <c r="F5" s="6">
+        <v>90</v>
+      </c>
+      <c r="G5" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="20"/>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="8" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -4944,16 +4935,16 @@
       <c r="E6" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F6" s="16">
-        <v>90</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="F6" s="6">
+        <v>90</v>
+      </c>
+      <c r="G6" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="20"/>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="8" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -4965,52 +4956,52 @@
       <c r="E7" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="16">
-        <v>90</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="F7" s="6">
+        <v>90</v>
+      </c>
+      <c r="G7" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="20"/>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="15" t="s">
         <v>231</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="13">
         <v>8</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="20"/>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="15" t="s">
         <v>232</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F9" s="24">
+      <c r="F9" s="13">
         <v>8</v>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="13">
         <v>11</v>
       </c>
     </row>
@@ -5018,7 +5009,7 @@
       <c r="A10" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -5030,16 +5021,16 @@
       <c r="E10" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F10" s="16">
-        <v>135</v>
-      </c>
-      <c r="G10" s="11">
+      <c r="F10" s="6">
+        <v>135</v>
+      </c>
+      <c r="G10" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="20"/>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -5051,16 +5042,16 @@
       <c r="E11" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F11" s="16">
-        <v>135</v>
-      </c>
-      <c r="G11" s="11">
+      <c r="F11" s="6">
+        <v>135</v>
+      </c>
+      <c r="G11" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="20"/>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="8" t="s">
         <v>5</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -5072,16 +5063,16 @@
       <c r="E12" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F12" s="16">
-        <v>135</v>
-      </c>
-      <c r="G12" s="11">
+      <c r="F12" s="6">
+        <v>135</v>
+      </c>
+      <c r="G12" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="20"/>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -5093,16 +5084,16 @@
       <c r="E13" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F13" s="16">
-        <v>90</v>
-      </c>
-      <c r="G13" s="11">
+      <c r="F13" s="6">
+        <v>90</v>
+      </c>
+      <c r="G13" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="20"/>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -5114,16 +5105,16 @@
       <c r="E14" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F14" s="16">
-        <v>90</v>
-      </c>
-      <c r="G14" s="11">
+      <c r="F14" s="6">
+        <v>90</v>
+      </c>
+      <c r="G14" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="20"/>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="8" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -5135,16 +5126,16 @@
       <c r="E15" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F15" s="16">
-        <v>90</v>
-      </c>
-      <c r="G15" s="11">
+      <c r="F15" s="6">
+        <v>90</v>
+      </c>
+      <c r="G15" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="20"/>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="8" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -5156,52 +5147,52 @@
       <c r="E16" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F16" s="16">
-        <v>90</v>
-      </c>
-      <c r="G16" s="11">
+      <c r="F16" s="6">
+        <v>90</v>
+      </c>
+      <c r="G16" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="20"/>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="13">
         <v>8</v>
       </c>
-      <c r="G17" s="24">
+      <c r="G17" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="20"/>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="26" t="s">
+      <c r="C18" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="15" t="s">
         <v>242</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="13">
         <v>8</v>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="13">
         <v>11</v>
       </c>
     </row>
@@ -5209,7 +5200,7 @@
       <c r="A19" s="20" t="s">
         <v>243</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -5221,16 +5212,16 @@
       <c r="E19" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F19" s="16">
-        <v>135</v>
-      </c>
-      <c r="G19" s="11">
+      <c r="F19" s="6">
+        <v>135</v>
+      </c>
+      <c r="G19" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="20"/>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -5242,16 +5233,16 @@
       <c r="E20" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F20" s="16">
-        <v>135</v>
-      </c>
-      <c r="G20" s="11">
+      <c r="F20" s="6">
+        <v>135</v>
+      </c>
+      <c r="G20" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="20"/>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="8" t="s">
         <v>5</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -5263,16 +5254,16 @@
       <c r="E21" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F21" s="16">
-        <v>135</v>
-      </c>
-      <c r="G21" s="11">
+      <c r="F21" s="6">
+        <v>135</v>
+      </c>
+      <c r="G21" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="20"/>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -5284,16 +5275,16 @@
       <c r="E22" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F22" s="16">
-        <v>90</v>
-      </c>
-      <c r="G22" s="11">
+      <c r="F22" s="6">
+        <v>90</v>
+      </c>
+      <c r="G22" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="20"/>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -5305,16 +5296,16 @@
       <c r="E23" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F23" s="16">
-        <v>90</v>
-      </c>
-      <c r="G23" s="11">
+      <c r="F23" s="6">
+        <v>90</v>
+      </c>
+      <c r="G23" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="20"/>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="8" t="s">
         <v>11</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -5326,16 +5317,16 @@
       <c r="E24" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F24" s="16">
-        <v>90</v>
-      </c>
-      <c r="G24" s="11">
+      <c r="F24" s="6">
+        <v>90</v>
+      </c>
+      <c r="G24" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="20"/>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="8" t="s">
         <v>13</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -5347,52 +5338,52 @@
       <c r="E25" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F25" s="16">
-        <v>90</v>
-      </c>
-      <c r="G25" s="11">
+      <c r="F25" s="6">
+        <v>90</v>
+      </c>
+      <c r="G25" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="20"/>
-      <c r="B26" s="27" t="s">
+      <c r="B26" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="D26" s="26" t="s">
+      <c r="D26" s="15" t="s">
         <v>251</v>
       </c>
-      <c r="E26" s="26" t="s">
+      <c r="E26" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F26" s="24">
+      <c r="F26" s="13">
         <v>8</v>
       </c>
-      <c r="G26" s="24">
+      <c r="G26" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="20"/>
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="D27" s="26" t="s">
+      <c r="D27" s="15" t="s">
         <v>252</v>
       </c>
-      <c r="E27" s="26" t="s">
+      <c r="E27" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F27" s="24">
+      <c r="F27" s="13">
         <v>8</v>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="13">
         <v>11</v>
       </c>
     </row>
@@ -5400,7 +5391,7 @@
       <c r="A28" s="20" t="s">
         <v>253</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -5412,16 +5403,16 @@
       <c r="E28" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="16">
-        <v>135</v>
-      </c>
-      <c r="G28" s="11">
+      <c r="F28" s="6">
+        <v>135</v>
+      </c>
+      <c r="G28" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="20"/>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -5433,16 +5424,16 @@
       <c r="E29" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F29" s="16">
-        <v>135</v>
-      </c>
-      <c r="G29" s="11">
+      <c r="F29" s="6">
+        <v>135</v>
+      </c>
+      <c r="G29" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="20"/>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="8" t="s">
         <v>5</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -5454,16 +5445,16 @@
       <c r="E30" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F30" s="16">
-        <v>135</v>
-      </c>
-      <c r="G30" s="11">
+      <c r="F30" s="6">
+        <v>135</v>
+      </c>
+      <c r="G30" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="20"/>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -5475,16 +5466,16 @@
       <c r="E31" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F31" s="16">
-        <v>90</v>
-      </c>
-      <c r="G31" s="11">
+      <c r="F31" s="6">
+        <v>90</v>
+      </c>
+      <c r="G31" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="20"/>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -5496,16 +5487,16 @@
       <c r="E32" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F32" s="16">
-        <v>90</v>
-      </c>
-      <c r="G32" s="11">
+      <c r="F32" s="6">
+        <v>90</v>
+      </c>
+      <c r="G32" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="20"/>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="8" t="s">
         <v>11</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -5517,16 +5508,16 @@
       <c r="E33" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F33" s="16">
-        <v>90</v>
-      </c>
-      <c r="G33" s="11">
+      <c r="F33" s="6">
+        <v>90</v>
+      </c>
+      <c r="G33" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="20"/>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="8" t="s">
         <v>13</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -5538,52 +5529,52 @@
       <c r="E34" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F34" s="16">
-        <v>90</v>
-      </c>
-      <c r="G34" s="11">
+      <c r="F34" s="6">
+        <v>90</v>
+      </c>
+      <c r="G34" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="20"/>
-      <c r="B35" s="27" t="s">
+      <c r="B35" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C35" s="26" t="s">
+      <c r="C35" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D35" s="26" t="s">
+      <c r="D35" s="15" t="s">
         <v>261</v>
       </c>
-      <c r="E35" s="26" t="s">
+      <c r="E35" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F35" s="24">
+      <c r="F35" s="13">
         <v>8</v>
       </c>
-      <c r="G35" s="24">
+      <c r="G35" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="20"/>
-      <c r="B36" s="27" t="s">
+      <c r="B36" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C36" s="26" t="s">
+      <c r="C36" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="D36" s="26" t="s">
+      <c r="D36" s="15" t="s">
         <v>262</v>
       </c>
-      <c r="E36" s="26" t="s">
+      <c r="E36" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F36" s="24">
+      <c r="F36" s="13">
         <v>8</v>
       </c>
-      <c r="G36" s="24">
+      <c r="G36" s="13">
         <v>11</v>
       </c>
     </row>
@@ -5591,7 +5582,7 @@
       <c r="A37" s="20" t="s">
         <v>263</v>
       </c>
-      <c r="B37" s="10" t="s">
+      <c r="B37" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C37" s="2" t="s">
@@ -5603,16 +5594,16 @@
       <c r="E37" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F37" s="16">
-        <v>135</v>
-      </c>
-      <c r="G37" s="11">
+      <c r="F37" s="6">
+        <v>135</v>
+      </c>
+      <c r="G37" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="20"/>
-      <c r="B38" s="10" t="s">
+      <c r="B38" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C38" s="2" t="s">
@@ -5624,16 +5615,16 @@
       <c r="E38" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F38" s="16">
-        <v>135</v>
-      </c>
-      <c r="G38" s="11">
+      <c r="F38" s="6">
+        <v>135</v>
+      </c>
+      <c r="G38" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="20"/>
-      <c r="B39" s="10" t="s">
+      <c r="B39" s="8" t="s">
         <v>5</v>
       </c>
       <c r="C39" s="2" t="s">
@@ -5645,16 +5636,16 @@
       <c r="E39" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F39" s="16">
-        <v>135</v>
-      </c>
-      <c r="G39" s="11">
+      <c r="F39" s="6">
+        <v>135</v>
+      </c>
+      <c r="G39" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="20"/>
-      <c r="B40" s="10" t="s">
+      <c r="B40" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C40" s="2" t="s">
@@ -5666,16 +5657,16 @@
       <c r="E40" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F40" s="16">
-        <v>90</v>
-      </c>
-      <c r="G40" s="11">
+      <c r="F40" s="6">
+        <v>90</v>
+      </c>
+      <c r="G40" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="20"/>
-      <c r="B41" s="10" t="s">
+      <c r="B41" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C41" s="2" t="s">
@@ -5687,16 +5678,16 @@
       <c r="E41" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F41" s="16">
-        <v>90</v>
-      </c>
-      <c r="G41" s="11">
+      <c r="F41" s="6">
+        <v>90</v>
+      </c>
+      <c r="G41" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="20"/>
-      <c r="B42" s="10" t="s">
+      <c r="B42" s="8" t="s">
         <v>11</v>
       </c>
       <c r="C42" s="2" t="s">
@@ -5708,16 +5699,16 @@
       <c r="E42" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F42" s="16">
-        <v>90</v>
-      </c>
-      <c r="G42" s="11">
+      <c r="F42" s="6">
+        <v>90</v>
+      </c>
+      <c r="G42" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="20"/>
-      <c r="B43" s="10" t="s">
+      <c r="B43" s="8" t="s">
         <v>13</v>
       </c>
       <c r="C43" s="2" t="s">
@@ -5729,52 +5720,52 @@
       <c r="E43" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F43" s="16">
-        <v>90</v>
-      </c>
-      <c r="G43" s="11">
+      <c r="F43" s="6">
+        <v>90</v>
+      </c>
+      <c r="G43" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="20"/>
-      <c r="B44" s="27" t="s">
+      <c r="B44" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C44" s="26" t="s">
+      <c r="C44" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="D44" s="26" t="s">
+      <c r="D44" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="E44" s="26" t="s">
+      <c r="E44" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F44" s="24">
+      <c r="F44" s="13">
         <v>8</v>
       </c>
-      <c r="G44" s="24">
+      <c r="G44" s="13">
         <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="20"/>
-      <c r="B45" s="27" t="s">
+      <c r="B45" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C45" s="26" t="s">
+      <c r="C45" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="D45" s="26" t="s">
+      <c r="D45" s="15" t="s">
         <v>272</v>
       </c>
-      <c r="E45" s="26" t="s">
+      <c r="E45" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="F45" s="24">
+      <c r="F45" s="13">
         <v>8</v>
       </c>
-      <c r="G45" s="24">
+      <c r="G45" s="13">
         <v>11</v>
       </c>
     </row>
@@ -5800,7 +5791,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5814,7 +5805,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -5823,15 +5814,15 @@
         <v>125</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F1" s="7">
+      <c r="F1" s="6">
         <v>110</v>
       </c>
-      <c r="G1" s="7">
+      <c r="G1" s="6">
         <v>120</v>
       </c>
     </row>
@@ -5844,15 +5835,15 @@
         <v>126</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="6">
         <v>110</v>
       </c>
-      <c r="G2" s="11">
+      <c r="G2" s="6">
         <v>120</v>
       </c>
     </row>
@@ -5865,57 +5856,57 @@
         <v>127</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F3" s="16">
+      <c r="F3" s="6">
         <v>110</v>
       </c>
-      <c r="G3" s="11">
+      <c r="G3" s="6">
         <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="18"/>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>128</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="6">
         <v>75</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="6">
         <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="19"/>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>129</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="6">
         <v>75</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="6">
         <v>85</v>
       </c>
     </row>
@@ -5923,169 +5914,169 @@
       <c r="A6" s="21" t="s">
         <v>273</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>312</v>
+      <c r="B6" s="9" t="s">
+        <v>311</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="9" t="s">
         <v>274</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="11">
         <v>80</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="22"/>
-      <c r="B7" s="12" t="s">
-        <v>313</v>
+      <c r="B7" s="9" t="s">
+        <v>312</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="9" t="s">
         <v>275</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="22"/>
-      <c r="B8" s="12" t="s">
-        <v>314</v>
+      <c r="B8" s="9" t="s">
+        <v>313</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="9" t="s">
         <v>276</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="22"/>
-      <c r="B9" s="12" t="s">
-        <v>315</v>
+      <c r="B9" s="9" t="s">
+        <v>314</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="9" t="s">
         <v>277</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G9" s="14">
+      <c r="G9" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="22"/>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="10" t="s">
         <v>278</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="9" t="s">
         <v>279</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="22"/>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="10" t="s">
         <v>280</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="9" t="s">
         <v>281</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F11" s="14">
+      <c r="F11" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G11" s="14">
+      <c r="G11" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="22"/>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="10" t="s">
         <v>282</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="9" t="s">
         <v>283</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F12" s="14">
+      <c r="F12" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G12" s="14">
+      <c r="G12" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="23"/>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="10" t="s">
         <v>284</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="9" t="s">
         <v>285</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F13" s="14">
+      <c r="F13" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G13" s="14">
+      <c r="G13" s="11">
         <v>90</v>
       </c>
     </row>
@@ -6093,368 +6084,368 @@
       <c r="A14" s="21" t="s">
         <v>286</v>
       </c>
-      <c r="B14" s="13" t="s">
-        <v>316</v>
+      <c r="B14" s="10" t="s">
+        <v>315</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="9" t="s">
         <v>287</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="22"/>
-      <c r="B15" s="13" t="s">
-        <v>317</v>
+      <c r="B15" s="10" t="s">
+        <v>316</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="9" t="s">
         <v>288</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="22"/>
-      <c r="B16" s="13" t="s">
-        <v>318</v>
+      <c r="B16" s="10" t="s">
+        <v>317</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="9" t="s">
         <v>289</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F16" s="14">
+      <c r="F16" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G16" s="14">
+      <c r="G16" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="22"/>
-      <c r="B17" s="13" t="s">
-        <v>319</v>
+      <c r="B17" s="10" t="s">
+        <v>318</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="9" t="s">
         <v>290</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F17" s="14">
+      <c r="F17" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G17" s="14">
+      <c r="G17" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="22"/>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="10" t="s">
         <v>278</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="9" t="s">
         <v>291</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F18" s="14">
+      <c r="F18" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G18" s="14">
+      <c r="G18" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="22"/>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="10" t="s">
         <v>280</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="9" t="s">
         <v>292</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F19" s="14">
+      <c r="F19" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G19" s="14">
+      <c r="G19" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="22"/>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="10" t="s">
         <v>282</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="D20" s="12" t="s">
-        <v>293</v>
+      <c r="D20" s="9" t="s">
+        <v>320</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F20" s="14">
+      <c r="F20" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G20" s="14">
+      <c r="G20" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="23"/>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="10" t="s">
         <v>284</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D21" s="12" t="s">
-        <v>294</v>
+      <c r="D21" s="9" t="s">
+        <v>293</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F21" s="14">
+      <c r="F21" s="11">
         <v>79.400000000000006</v>
       </c>
-      <c r="G21" s="14">
+      <c r="G21" s="11">
         <v>90</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
-        <v>311</v>
-      </c>
-      <c r="B22" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="D22" s="12" t="s">
-        <v>295</v>
+      <c r="D22" s="9" t="s">
+        <v>294</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F22" s="14">
-        <v>135</v>
-      </c>
-      <c r="G22" s="14">
+      <c r="F22" s="11">
+        <v>135</v>
+      </c>
+      <c r="G22" s="11">
         <v>145</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="22"/>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D23" s="12" t="s">
-        <v>296</v>
+      <c r="D23" s="9" t="s">
+        <v>295</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F23" s="16">
-        <v>135</v>
-      </c>
-      <c r="G23" s="16">
+      <c r="F23" s="6">
+        <v>135</v>
+      </c>
+      <c r="G23" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="22"/>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D24" s="12" t="s">
-        <v>297</v>
+      <c r="D24" s="9" t="s">
+        <v>296</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F24" s="16">
-        <v>135</v>
-      </c>
-      <c r="G24" s="16">
+      <c r="F24" s="6">
+        <v>135</v>
+      </c>
+      <c r="G24" s="6">
         <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="22"/>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D25" s="12" t="s">
-        <v>298</v>
+      <c r="D25" s="9" t="s">
+        <v>297</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F25" s="16">
-        <v>90</v>
-      </c>
-      <c r="G25" s="16">
+      <c r="F25" s="6">
+        <v>90</v>
+      </c>
+      <c r="G25" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="22"/>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D26" s="12" t="s">
-        <v>299</v>
+      <c r="D26" s="9" t="s">
+        <v>298</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F26" s="16">
-        <v>90</v>
-      </c>
-      <c r="G26" s="16">
+      <c r="F26" s="6">
+        <v>90</v>
+      </c>
+      <c r="G26" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="22"/>
-      <c r="B27" s="8" t="s">
-        <v>310</v>
+      <c r="B27" s="7" t="s">
+        <v>309</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="D27" s="12" t="s">
-        <v>300</v>
+      <c r="D27" s="9" t="s">
+        <v>299</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F27" s="16">
-        <v>90</v>
-      </c>
-      <c r="G27" s="16">
+      <c r="F27" s="6">
+        <v>90</v>
+      </c>
+      <c r="G27" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="22"/>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="D28" s="12" t="s">
-        <v>301</v>
+      <c r="D28" s="9" t="s">
+        <v>300</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="16">
-        <v>90</v>
-      </c>
-      <c r="G28" s="16">
+      <c r="F28" s="6">
+        <v>90</v>
+      </c>
+      <c r="G28" s="6">
         <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="22"/>
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="9" t="s">
         <v>15</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="D29" s="12" t="s">
-        <v>302</v>
+      <c r="D29" s="9" t="s">
+        <v>301</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="F29" s="7">
+      <c r="F29" s="6">
         <v>79.400000000000006</v>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="6">
         <v>90</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="23"/>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="D30" s="12" t="s">
-        <v>303</v>
+      <c r="D30" s="9" t="s">
+        <v>302</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="6">
         <v>79.400000000000006</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="6">
         <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="G31" s="7" t="s">
+      <c r="G31" s="6" t="s">
         <v>164</v>
       </c>
     </row>

</xml_diff>

<commit_message>
create UI page MBA
</commit_message>
<xml_diff>
--- a/public/TagDongCoVoi.xlsx
+++ b/public/TagDongCoVoi.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E63780-918B-4A05-B09C-757AD3C97C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B345BE7-059C-4F11-9120-41AE23859E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoVoi1" sheetId="1" r:id="rId1"/>
@@ -14,6 +14,7 @@
     <sheet name="Dolomit1" sheetId="4" r:id="rId4"/>
     <sheet name="Dolomit2" sheetId="5" r:id="rId5"/>
     <sheet name="LoVoiQuay" sheetId="6" r:id="rId6"/>
+    <sheet name="ThanhPham" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="350">
   <si>
     <t>Nhiệt độ pha A</t>
   </si>
@@ -988,13 +989,100 @@
   </si>
   <si>
     <t>Động cơ chính Lò vôi quay quay</t>
+  </si>
+  <si>
+    <t>Dòng điện động cơ gầu nâng 2 thành phẩm lò vôi</t>
+  </si>
+  <si>
+    <t>Dòng điện máy nghiền thành phẩm lò vôi 3</t>
+  </si>
+  <si>
+    <t>Dòng điện máy nghiền thành phẩm lò vôi 2</t>
+  </si>
+  <si>
+    <t>Dòng điện máy nghiền thành phẩm lò vôi 1</t>
+  </si>
+  <si>
+    <t>Gầu nâng đá loại dolomit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Dòng điện động cơ gầu nâng 1 thành phẩm dolomit</t>
+  </si>
+  <si>
+    <t>Dòng điện động cơ gầu nâng 2 thành phẩm dolomit</t>
+  </si>
+  <si>
+    <t>Máy nghiền 1 thành phẩm dolomit 1</t>
+  </si>
+  <si>
+    <t>Máy nghiền 1 thành phẩm dolomit 2</t>
+  </si>
+  <si>
+    <t>Dòng điện động cơ gầu nâng 1 thành phẩm lò vôi quay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Dòng điện động cơ gầu nâng 2 thành phẩm lò vôi quay</t>
+  </si>
+  <si>
+    <t>DONG_DIEN_GAUNANGTHANHPHAM_3_VOI</t>
+  </si>
+  <si>
+    <t>DONG_DIEN_GAUNANGTHANHPHAM_2_VOI</t>
+  </si>
+  <si>
+    <t>DONG_DIEN_GAUNANGTHANHPHAM_1_VOI</t>
+  </si>
+  <si>
+    <t>finished_product_3#_cusher_current_feedback</t>
+  </si>
+  <si>
+    <t>finished_product_2#_cusher_current_feedback</t>
+  </si>
+  <si>
+    <t>finished_product_1#_cusher_current_feedback</t>
+  </si>
+  <si>
+    <t>DONG_DIEN_GAU_NANG_DA_LOAI_DLM</t>
+  </si>
+  <si>
+    <t>DONG_DIEN_GAU_NANG_1_TP_DLM</t>
+  </si>
+  <si>
+    <t>DONG_DIEN_GAU_NANG_2_TP_DLM</t>
+  </si>
+  <si>
+    <t>Kiln_finised_product_1#_crusher_current_feedback</t>
+  </si>
+  <si>
+    <t>Kiln_finised_product_2#_crusher_current_feedback</t>
+  </si>
+  <si>
+    <t>AI_Product_1#_bucket_elevator_current_display</t>
+  </si>
+  <si>
+    <t>AI_Product_2#_bucket_elevator_current_display</t>
+  </si>
+  <si>
+    <t>Khu thành phẩm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Dòng điện động cơ gầu nâng 1 thành phẩm lò vôi</t>
+  </si>
+  <si>
+    <t>Dòng điện động cơ gầu nâng 3 thành phẩm lò vôi</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Đơn vị</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1051,6 +1139,24 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1158,7 +1264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1212,6 +1318,17 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6810,4 +6927,262 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEB0F74A-32E1-4A2C-AE99-6B8DCF1A1100}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.5703125" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" customWidth="1"/>
+    <col min="4" max="4" width="72.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
+        <v>345</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>346</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>334</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+    </row>
+    <row r="2" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="23"/>
+      <c r="B2" s="24" t="s">
+        <v>321</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>333</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+    </row>
+    <row r="3" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="23"/>
+      <c r="B3" s="24" t="s">
+        <v>347</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>332</v>
+      </c>
+      <c r="E3" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+    </row>
+    <row r="4" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="23"/>
+      <c r="B4" s="24" t="s">
+        <v>324</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>337</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+    </row>
+    <row r="5" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="23"/>
+      <c r="B5" s="24" t="s">
+        <v>323</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="E5" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+    </row>
+    <row r="6" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="23"/>
+      <c r="B6" s="24" t="s">
+        <v>322</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>335</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+    </row>
+    <row r="7" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="23"/>
+      <c r="B7" s="25" t="s">
+        <v>325</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>338</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+    </row>
+    <row r="8" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="23"/>
+      <c r="B8" s="24" t="s">
+        <v>326</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+    </row>
+    <row r="9" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="23"/>
+      <c r="B9" s="25" t="s">
+        <v>327</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>340</v>
+      </c>
+      <c r="E9" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+    </row>
+    <row r="10" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="23"/>
+      <c r="B10" s="24" t="s">
+        <v>328</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>341</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+    </row>
+    <row r="11" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="23"/>
+      <c r="B11" s="25" t="s">
+        <v>329</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>342</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+    </row>
+    <row r="12" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="23"/>
+      <c r="B12" s="25" t="s">
+        <v>330</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>343</v>
+      </c>
+      <c r="E12" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+    </row>
+    <row r="13" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="23"/>
+      <c r="B13" s="25" t="s">
+        <v>331</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>344</v>
+      </c>
+      <c r="E13" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E14" s="22" t="s">
+        <v>349</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>152</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:A13"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>